<commit_message>
Version 2.0: Update latest signal results
</commit_message>
<xml_diff>
--- a/results/latest_signals.xlsx
+++ b/results/latest_signals.xlsx
@@ -694,10 +694,10 @@
         <v>62.22684703433923</v>
       </c>
       <c r="I4" t="n">
-        <v>10.91955270559083</v>
+        <v>10.91955270557628</v>
       </c>
       <c r="J4" t="n">
-        <v>-10.80961385649457</v>
+        <v>-10.80961385651522</v>
       </c>
       <c r="K4" t="n">
         <v>137.5714285714286</v>
@@ -766,10 +766,10 @@
         <v>53.05263157894736</v>
       </c>
       <c r="I5" t="n">
-        <v>23.31215952163075</v>
+        <v>23.3121595216362</v>
       </c>
       <c r="J5" t="n">
-        <v>15.7653577149812</v>
+        <v>15.76535771498861</v>
       </c>
       <c r="K5" t="n">
         <v>76.28571428571429</v>
@@ -910,10 +910,10 @@
         <v>57.11340206185567</v>
       </c>
       <c r="I7" t="n">
-        <v>21.52534935291669</v>
+        <v>21.52534935291033</v>
       </c>
       <c r="J7" t="n">
-        <v>7.823164239502628</v>
+        <v>7.823164239493314</v>
       </c>
       <c r="K7" t="n">
         <v>60.42857142857143</v>
@@ -1198,10 +1198,10 @@
         <v>40.15887025595763</v>
       </c>
       <c r="I11" t="n">
-        <v>-217.0396306074163</v>
+        <v>-217.0396306074199</v>
       </c>
       <c r="J11" t="n">
-        <v>-177.0751115275796</v>
+        <v>-177.0751115275854</v>
       </c>
       <c r="K11" t="n">
         <v>436.4285714285714</v>

</xml_diff>